<commit_message>
Updated peoplesoft version and added exception handling in Peoplesoft flow and config file
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55648C\Documents\SOK_GIT\P0001_090_PayCyleQueries_Dispatcher\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D312EF-5BAD-4417-BBDE-F8A28A451094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57137EC4-2F09-4056-81F5-701E3414CFBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="258">
   <si>
     <t>Name</t>
   </si>
@@ -102,11 +102,11 @@
   </si>
   <si>
     <t>Logging field which allows grouping of log data of two or more subprocesses under the same business process name</t>
-    <phoneticPr fontId="14"/>
+    <phoneticPr fontId="15"/>
   </si>
   <si>
     <t>OrchestratorQueueName</t>
-    <phoneticPr fontId="14"/>
+    <phoneticPr fontId="15"/>
   </si>
   <si>
     <t>Must be 0 if working with Orchestrator queues. If &gt; 0, the robot will retry the same transaction which failed with a system exception. Must be an integer value.</t>
@@ -876,18 +876,46 @@
     <t>This is the process Name value value for Process Monitor refresh</t>
   </si>
   <si>
-    <t>DEV</t>
+    <t>SE_8</t>
+  </si>
+  <si>
+    <t>SE_8: {Element} value could not be entered in Process Monitor</t>
+  </si>
+  <si>
+    <t>Text value entry failed in Process Monitor for {Process Name} Process</t>
+  </si>
+  <si>
+    <t>Hi Statewide Accounting Team,&lt;br&gt;&lt;br&gt;
+The error occurred while updating filters in Process Monitor. The error details are as follows&lt;br&gt;&lt;br&gt;
+&lt;u&gt;Error Details:&lt;/u&gt; {Exception Details}&lt;br&gt;&lt;br&gt;
+Thanks,&lt;br&gt;</t>
+  </si>
+  <si>
+    <t>RetryNumberProcessMonitorFilter</t>
+  </si>
+  <si>
+    <t>The number of time the filters should be input to update the process monitor view. Must be an integer &gt;=1</t>
+  </si>
+  <si>
+    <t>PROD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1073,64 +1101,67 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1143,6 +1174,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1537,8 +1571,8 @@
         <v>29</v>
       </c>
       <c r="B4" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>30</v>
@@ -1576,8 +1610,8 @@
         <v>197</v>
       </c>
       <c r="B9" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>198</v>
@@ -1592,8 +1626,8 @@
         <v>95</v>
       </c>
       <c r="B11" s="2" t="str">
-        <f>Constants!$B$19</f>
-        <v>DEV</v>
+        <f>Constants!$B$20</f>
+        <v>PROD</v>
       </c>
       <c r="C11" t="s">
         <v>96</v>
@@ -2654,7 +2688,7 @@
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="14"/>
+  <phoneticPr fontId="15"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2662,7 +2696,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Z989"/>
+  <dimension ref="A1:Z990"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
@@ -2837,28 +2871,38 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="14.25" customHeight="1"/>
-    <row r="18" spans="1:3" ht="45">
-      <c r="A18" t="s">
+    <row r="17" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>255</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1"/>
+    <row r="19" spans="1:3" ht="45">
+      <c r="A19" t="s">
         <v>38</v>
       </c>
-      <c r="B18" t="b">
+      <c r="B19" t="b">
         <v>0</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
-      <c r="A19" t="s">
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
         <v>212</v>
       </c>
-      <c r="B19" t="s">
-        <v>251</v>
-      </c>
-      <c r="C19" s="3"/>
-    </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1"/>
+      <c r="B20" t="s">
+        <v>257</v>
+      </c>
+      <c r="C20" s="3"/>
+    </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="23" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="24" spans="1:3" ht="14.25" customHeight="1"/>
@@ -3827,8 +3871,9 @@
     <row r="987" ht="14.25" customHeight="1"/>
     <row r="988" ht="14.25" customHeight="1"/>
     <row r="989" ht="14.25" customHeight="1"/>
+    <row r="990" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="14"/>
+  <phoneticPr fontId="15"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3889,8 +3934,8 @@
         <v>49</v>
       </c>
       <c r="C2" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
@@ -3901,8 +3946,8 @@
         <v>50</v>
       </c>
       <c r="C3" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -3913,8 +3958,8 @@
         <v>51</v>
       </c>
       <c r="C4" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D4" t="s">
         <v>240</v>
@@ -3928,8 +3973,8 @@
         <v>59</v>
       </c>
       <c r="C5" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>211</v>
@@ -3943,8 +3988,8 @@
         <v>71</v>
       </c>
       <c r="C6" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>82</v>
@@ -3958,8 +4003,8 @@
         <v>73</v>
       </c>
       <c r="C7" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>82</v>
@@ -3973,8 +4018,8 @@
         <v>76</v>
       </c>
       <c r="C8" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>83</v>
@@ -3988,8 +4033,8 @@
         <v>77</v>
       </c>
       <c r="C9" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>83</v>
@@ -4003,8 +4048,8 @@
         <v>80</v>
       </c>
       <c r="C10" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>84</v>
@@ -4018,8 +4063,8 @@
         <v>81</v>
       </c>
       <c r="C11" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>84</v>
@@ -4033,8 +4078,8 @@
         <v>86</v>
       </c>
       <c r="C12" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>87</v>
@@ -4048,8 +4093,8 @@
         <v>89</v>
       </c>
       <c r="C13" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>90</v>
@@ -4063,8 +4108,8 @@
         <v>217</v>
       </c>
       <c r="C14" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>218</v>
@@ -4078,8 +4123,8 @@
         <v>100</v>
       </c>
       <c r="C15" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>101</v>
@@ -4093,8 +4138,8 @@
         <v>99</v>
       </c>
       <c r="C16" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>102</v>
@@ -4108,8 +4153,8 @@
         <v>104</v>
       </c>
       <c r="C17" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>105</v>
@@ -4123,8 +4168,8 @@
         <v>137</v>
       </c>
       <c r="C18" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>138</v>
@@ -4138,8 +4183,8 @@
         <v>141</v>
       </c>
       <c r="C19" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>143</v>
@@ -4153,8 +4198,8 @@
         <v>142</v>
       </c>
       <c r="C20" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>144</v>
@@ -4168,8 +4213,8 @@
         <v>157</v>
       </c>
       <c r="C21" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>163</v>
@@ -4183,8 +4228,8 @@
         <v>162</v>
       </c>
       <c r="C22" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>164</v>
@@ -4198,8 +4243,8 @@
         <v>158</v>
       </c>
       <c r="C23" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>165</v>
@@ -4213,8 +4258,8 @@
         <v>159</v>
       </c>
       <c r="C24" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>166</v>
@@ -4228,8 +4273,8 @@
         <v>160</v>
       </c>
       <c r="C25" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>167</v>
@@ -4243,8 +4288,8 @@
         <v>161</v>
       </c>
       <c r="C26" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>168</v>
@@ -4258,8 +4303,8 @@
         <v>169</v>
       </c>
       <c r="C27" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>175</v>
@@ -4273,8 +4318,8 @@
         <v>170</v>
       </c>
       <c r="C28" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>176</v>
@@ -4288,8 +4333,8 @@
         <v>171</v>
       </c>
       <c r="C29" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>177</v>
@@ -4303,8 +4348,8 @@
         <v>172</v>
       </c>
       <c r="C30" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>178</v>
@@ -4318,8 +4363,8 @@
         <v>173</v>
       </c>
       <c r="C31" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>179</v>
@@ -4333,8 +4378,8 @@
         <v>174</v>
       </c>
       <c r="C32" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>180</v>
@@ -4348,8 +4393,8 @@
         <v>182</v>
       </c>
       <c r="C33" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>183</v>
@@ -4363,8 +4408,8 @@
         <v>185</v>
       </c>
       <c r="C34" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>186</v>
@@ -4378,8 +4423,8 @@
         <v>188</v>
       </c>
       <c r="C35" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>189</v>
@@ -4393,8 +4438,8 @@
         <v>219</v>
       </c>
       <c r="C36" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>221</v>
@@ -4408,8 +4453,8 @@
         <v>223</v>
       </c>
       <c r="C37" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>239</v>
@@ -4423,8 +4468,8 @@
         <v>225</v>
       </c>
       <c r="C38" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D38" t="s">
         <v>238</v>
@@ -4438,8 +4483,8 @@
         <v>232</v>
       </c>
       <c r="C39" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D39" t="s">
         <v>235</v>
@@ -4453,8 +4498,8 @@
         <v>233</v>
       </c>
       <c r="C40" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D40" t="s">
         <v>236</v>
@@ -4468,8 +4513,8 @@
         <v>234</v>
       </c>
       <c r="C41" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D41" t="s">
         <v>237</v>
@@ -4483,8 +4528,8 @@
         <v>247</v>
       </c>
       <c r="C42" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D42" t="s">
         <v>249</v>
@@ -4498,8 +4543,8 @@
         <v>248</v>
       </c>
       <c r="C43" s="2" t="str">
-        <f>_xlfn.CONCAT(Constants!$B$19,"/P001_090_PayCycleQueries")</f>
-        <v>DEV/P001_090_PayCycleQueries</v>
+        <f>_xlfn.CONCAT(Constants!$B$20,"/P001_090_PayCycleQueries")</f>
+        <v>PROD/P001_090_PayCycleQueries</v>
       </c>
       <c r="D43" t="s">
         <v>250</v>
@@ -5457,14 +5502,14 @@
     <row r="993" ht="14.25" customHeight="1"/>
     <row r="994" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="14"/>
+  <phoneticPr fontId="15"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CB048EB-7BC5-4528-AC4D-7EFC70AE54E8}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -5707,66 +5752,70 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="40.5" customHeight="1">
-      <c r="A10" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>132</v>
+    <row r="10" spans="1:8" ht="45" customHeight="1">
+      <c r="A10" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>252</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>209</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>123</v>
+        <v>111</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>253</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>254</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="10" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" ht="40.5" customHeight="1">
       <c r="A11" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="B11" s="15" t="s">
-        <v>133</v>
+        <v>114</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>132</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="9" t="s">
-        <v>117</v>
+      <c r="D11" s="24" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>123</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="G11" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="H11" s="8"/>
+      <c r="H11" s="13" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>115</v>
       </c>
       <c r="D12" s="8"/>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="9" t="s">
         <v>117</v>
       </c>
       <c r="F12" s="8" t="s">
@@ -5777,12 +5826,12 @@
       </c>
       <c r="H12" s="8"/>
     </row>
-    <row r="13" spans="1:8" ht="30">
+    <row r="13" spans="1:8">
       <c r="A13" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>135</v>
+        <v>119</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>134</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>115</v>
@@ -5799,15 +5848,37 @@
       </c>
       <c r="H13" s="8"/>
     </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
+    <row r="14" spans="1:8" ht="30">
+      <c r="A14" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="G14" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="H14" s="8"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="5"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>